<commit_message>
Asociación LG ↔ PCZ: elegir N° Novedad y Hora al cargar; hora de PCZ en el puntaje
- Carga: LG elige Fecha, Transcripción y Hora (opcional); PCZ elige
  Fecha, Descripción, N° Novedad (o "usar el número de fila del Excel")
  y Hora (opcional). Se sugieren por nombre. Se quita Página.
- La ayuda de N° Novedad aclara que es el valor que se junta con ";" en
  la hoja LG_asociado cuando un párrafo tiene varias novedades.
- La columna Hora de PCZ ahora suma al puntaje de cercanía horaria y se
  muestra en las tarjetas.
- PCZ de ejemplo con columna Hora; tests nuevos; README actualizado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HyHMnb383MqJUjAQYTPPyJ
</commit_message>
<xml_diff>
--- a/tests/ejemplos/PCZ_ejemplo.xlsx
+++ b/tests/ejemplos/PCZ_ejemplo.xlsx
@@ -49,9 +49,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,6 +437,11 @@
           <t>Nº Novedad</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -449,6 +455,9 @@
       <c r="C2" t="n">
         <v>1001</v>
       </c>
+      <c r="D2" s="2" t="n">
+        <v>0.3402777777777778</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -464,6 +473,11 @@
       <c r="C3" t="n">
         <v>1002</v>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -479,6 +493,9 @@
       <c r="C4" t="n">
         <v>1003</v>
       </c>
+      <c r="D4" s="2" t="n">
+        <v>0.6076388888888888</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -505,6 +522,9 @@
       <c r="C6" t="n">
         <v>1005</v>
       </c>
+      <c r="D6" s="2" t="n">
+        <v>0.125</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -520,6 +540,11 @@
       <c r="C7" t="n">
         <v>1006</v>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -589,6 +614,9 @@
       <c r="C12" t="n">
         <v>1011</v>
       </c>
+      <c r="D12" s="2" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -617,6 +645,9 @@
       <c r="C14" t="n">
         <v>1013</v>
       </c>
+      <c r="D14" s="2" t="n">
+        <v>0.9965277777777778</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -632,6 +663,11 @@
       <c r="C15" t="n">
         <v>1014</v>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -645,6 +681,9 @@
       <c r="C16" t="n">
         <v>1015</v>
       </c>
+      <c r="D16" s="2" t="n">
+        <v>0.4791666666666667</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -686,6 +725,11 @@
       <c r="C19" t="n">
         <v>1018</v>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -699,6 +743,9 @@
       <c r="C20" t="n">
         <v>1019</v>
       </c>
+      <c r="D20" s="2" t="n">
+        <v>0.8402777777777778</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -740,6 +787,11 @@
       <c r="C23" t="n">
         <v>1022</v>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>06:20</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -755,6 +807,9 @@
       <c r="C24" t="n">
         <v>1023</v>
       </c>
+      <c r="D24" s="2" t="n">
+        <v>0.2916666666666667</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -783,6 +838,9 @@
       <c r="C26" t="n">
         <v>1025</v>
       </c>
+      <c r="D26" s="2" t="n">
+        <v>0.4375</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -810,6 +868,9 @@
       </c>
       <c r="C28" t="n">
         <v>1027</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>0.5104166666666666</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Asociación LG ↔ PCZ: columnas Zona, VER, Falla, Comienzo de falla y Habilitación
Después de «Descripción», la hoja Asociaciones trae estas 5 columnas copiadas de PCZ tal como
vienen (si se unieron varias novedades, sus valores distintos con « | »). Se eligen al cargar
(se reconocen solas por nombre) y son opcionales: si el PCZ no las tiene, quedan vacías.
Fecha y hora con formato d/m/yyyy h:mm. El PCZ de ejemplo inventado trae estas columnas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HyHMnb383MqJUjAQYTPPyJ
</commit_message>
<xml_diff>
--- a/tests/ejemplos/PCZ_ejemplo.xlsx
+++ b/tests/ejemplos/PCZ_ejemplo.xlsx
@@ -16,9 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="166" formatCode="DD/MM/YYYY HH:MM"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,10 +50,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,6 +444,31 @@
           <t>Hora</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>VER</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Falla</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Comienzo de falla</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Habilitación</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -458,6 +485,27 @@
       <c r="D2" s="2" t="n">
         <v>0.3402777777777778</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Zona 3</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Barreras</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>45720.34027777778</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>45720.37152777778</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -478,6 +526,21 @@
           <t>09:12</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Zona 1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -496,6 +559,21 @@
       <c r="D4" s="2" t="n">
         <v>0.6076388888888888</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Zona 2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Vía</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -509,6 +587,27 @@
       <c r="C5" t="n">
         <v>1004</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Zona 3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Señalamiento</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>45720.61805555555</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>45720.64930555555</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -525,6 +624,27 @@
       <c r="D6" s="2" t="n">
         <v>0.125</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Zona 1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Barreras</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>45720.125</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>45720.15625</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -545,6 +665,21 @@
           <t>07:20</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Zona 2</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -558,6 +693,21 @@
       <c r="C8" t="n">
         <v>1007</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Zona 3</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Vía</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -571,6 +721,27 @@
       <c r="C9" t="n">
         <v>1008</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Zona 1</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Señalamiento</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>45720.66666666666</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>45720.69791666666</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -586,6 +757,21 @@
       <c r="C10" t="n">
         <v>1009</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Zona 2</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Barreras</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -599,6 +785,21 @@
       <c r="C11" t="n">
         <v>1010</v>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Zona 3</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -617,6 +818,21 @@
       <c r="D12" s="2" t="n">
         <v>0.5</v>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Zona 1</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Vía</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -630,6 +846,21 @@
       <c r="C13" t="n">
         <v>1012</v>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Zona 2</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Señalamiento</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -648,6 +879,21 @@
       <c r="D14" s="2" t="n">
         <v>0.9965277777777778</v>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Zona 3</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Barreras</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -668,6 +914,21 @@
           <t>10:00</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Zona 1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -684,6 +945,27 @@
       <c r="D16" s="2" t="n">
         <v>0.4791666666666667</v>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Zona 2</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Vía</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>45721.47916666666</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>45721.51041666666</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -697,6 +979,21 @@
       <c r="C17" t="n">
         <v>1016</v>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Zona 3</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Señalamiento</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -712,6 +1009,21 @@
       <c r="C18" t="n">
         <v>1017</v>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Zona 1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Barreras</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -730,6 +1042,27 @@
           <t>18:20</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Zona 2</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>45721.76388888889</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>45721.79513888889</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -746,6 +1079,21 @@
       <c r="D20" s="2" t="n">
         <v>0.8402777777777778</v>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Zona 3</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Vía</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -761,6 +1109,21 @@
       <c r="C21" t="n">
         <v>1020</v>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Zona 1</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Señalamiento</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -774,6 +1137,21 @@
       <c r="C22" t="n">
         <v>1021</v>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Zona 2</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Barreras</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -792,6 +1170,27 @@
           <t>06:20</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Zona 3</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>45722.26388888889</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>45722.29513888889</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -810,6 +1209,21 @@
       <c r="D24" s="2" t="n">
         <v>0.2916666666666667</v>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Zona 1</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Vía</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -825,6 +1239,21 @@
       <c r="C25" t="n">
         <v>1024</v>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Zona 2</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Señalamiento</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -841,6 +1270,27 @@
       <c r="D26" s="2" t="n">
         <v>0.4375</v>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Zona 3</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Barreras</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>45722.4375</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>45722.46875</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -856,6 +1306,21 @@
       <c r="C27" t="n">
         <v>1026</v>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Zona 1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -872,6 +1337,27 @@
       <c r="D28" s="2" t="n">
         <v>0.5104166666666666</v>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Zona 2</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Vía</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>45722.51041666666</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>45722.54166666666</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -885,6 +1371,21 @@
       <c r="C29" t="n">
         <v>1028</v>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Zona 3</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Señalamiento</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -900,6 +1401,21 @@
       <c r="C30" t="n">
         <v>1029</v>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Zona 1</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Barreras</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -914,6 +1430,21 @@
       </c>
       <c r="C31" t="n">
         <v>1030</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Zona 2</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>